<commit_message>
Corriger l'export : les relevés valables sur toute la fenêtre étaient ignorés
Les constats du Groupe B portent la semaine « S1-S8 » — Vérone, Marbella
et Lublin, dont l'absence de vol direct vaut sur les huit semaines. La
boucle d'export parcourait la liste figée S1..S8 et les sautait
silencieusement : trois lignes manquaient à l'onglet Relevés.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JiaPbp62K1ogGYZBH5Bg98
</commit_message>
<xml_diff>
--- a/Data/CouponKasher_grille_S1-S8.xlsx
+++ b/Data/CouponKasher_grille_S1-S8.xlsx
@@ -1925,7 +1925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M52"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -4796,6 +4796,151 @@
       <c r="M52" s="21" t="inlineStr">
         <is>
           <t>Blue Bird direct TLV-Bergame a 316 $, Sirmione a ~80 km. Hotels hors Booking</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>ורונה</t>
+        </is>
+      </c>
+      <c r="B53" s="11" t="inlineStr"/>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>S1-S8</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E53" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F53" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H53" s="18" t="n"/>
+      <c r="I53" s="18" t="n"/>
+      <c r="J53" s="17" t="n"/>
+      <c r="K53" s="17" t="n"/>
+      <c r="L53" s="17" t="inlineStr">
+        <is>
+          <t>aucun vol direct</t>
+        </is>
+      </c>
+      <c r="M53" s="21" t="inlineStr">
+        <is>
+          <t>zero resultat sur VRN et zero en interrogeant la ville, sur les huit semaines. Aucun hotel identifie par ailleurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>Marbella</t>
+        </is>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>AGP</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>S1-S8</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="18" t="n"/>
+      <c r="I54" s="18" t="n"/>
+      <c r="J54" s="17" t="n"/>
+      <c r="K54" s="17" t="n"/>
+      <c r="L54" s="17" t="inlineStr">
+        <is>
+          <t>aucun vol direct</t>
+        </is>
+      </c>
+      <c r="M54" s="21" t="inlineStr">
+        <is>
+          <t>zero resultat sur AGP et sur Malaga, sur les huit semaines. Le 'pas de direct structurel' de la reference est confirme</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>לובלין</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="inlineStr"/>
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>S1-S8</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F55" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H55" s="18" t="n"/>
+      <c r="I55" s="18" t="n"/>
+      <c r="J55" s="17" t="n"/>
+      <c r="K55" s="17" t="n"/>
+      <c r="L55" s="17" t="inlineStr">
+        <is>
+          <t>aucun vol direct</t>
+        </is>
+      </c>
+      <c r="M55" s="21" t="inlineStr">
+        <is>
+          <t>aucun direct TLV-Lublin. Divergence a trancher entre Hotel Ilan (reference promo) et Hotel Olive (site)</t>
         </is>
       </c>
     </row>

</xml_diff>